<commit_message>
Fix minor text issue
</commit_message>
<xml_diff>
--- a/sample/04_Python in Excelによるデータ分析/サンプルデータ+ソースコード/サンプル_従業員データ.xlsx
+++ b/sample/04_Python in Excelによるデータ分析/サンプルデータ+ソースコード/サンプル_従業員データ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28314"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://erringtonracsch-my.sharepoint.com/personal/a36769_365c_pro/Documents/Python in Excel入門/00_send/src/04_Python in Excelによるデータ分析/サンプルデータ+ソースコード/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4970633B-044A-4B12-B324-4A7FBDFB643B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{4970633B-044A-4B12-B324-4A7FBDFB643B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D6DD542-3734-417B-9DB7-92BF42ADD760}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{80A00C8E-7DBF-42A7-B663-1B4E4E97E1C9}"/>
+    <workbookView xWindow="28695" yWindow="11745" windowWidth="14610" windowHeight="15585" xr2:uid="{80A00C8E-7DBF-42A7-B663-1B4E4E97E1C9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -85,7 +85,7 @@
     </pythonScript>
     <pythonScript>
       <code># 正規表現のパターンを指定する
-email_pattern = "^([^\s@]+)@((outlook\.mail)|([e|g]?mail\.com))$"
+email_pattern = "^([^\s@]+)@((outlook\.mail)|([eg]?mail\.com))$"
 # 各メールアドレスが正規表現のパターンを満たしているか判定する
 df["メールアドレス"].str.match(email_pattern)</code>
     </pythonScript>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="I1" s="1" t="str" cm="1">
         <f t="array" ref="I1:I6">_xlfn._xlws.PY(3,0)</f>
-        <v>outlook.mail</v>
+        <v>email.com</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -4225,7 +4225,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="1" t="str">
-        <v>email.com</v>
+        <v>gmail.com</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -4251,7 +4251,7 @@
         <v>1</v>
       </c>
       <c r="I3" s="1" t="str">
-        <v>gnail.com</v>
+        <v>gmaill.com</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -4277,7 +4277,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="1" t="str">
-        <v>mail.com</v>
+        <v>gnail.com</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -4303,7 +4303,7 @@
         <v>1</v>
       </c>
       <c r="I5" s="1" t="str">
-        <v>gmail.com</v>
+        <v>mail.com</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -4329,7 +4329,7 @@
         <v>1</v>
       </c>
       <c r="I6" s="1" t="str">
-        <v>gmaill.com</v>
+        <v>outlook.mail</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>